<commit_message>
make well names optional
</commit_message>
<xml_diff>
--- a/excel_templates/tirtl_manifest_template.xlsx
+++ b/excel_templates/tirtl_manifest_template.xlsx
@@ -1210,12 +1210,12 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Optional plate coordinate for the well represented by the FASTQ. Paired R1/R2 files from the same well must share the same value when provided. Leave blank for raw-mode submissions containing only a FASTQ pair.</t>
+          <t>Optional plate coordinate for the well represented by the FASTQ. Use the zero-padded format A01 through P24. Paired R1/R2 files from the same well must share the same value when provided. Leave blank for raw-mode submissions containing only a FASTQ pair.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Plate coordinates A1 through P24</t>
+          <t>Plate coordinates A01 through P24</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1225,7 +1225,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>A01</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr"/>

</xml_diff>